<commit_message>
Update historical price analysis 2026-04
</commit_message>
<xml_diff>
--- a/outputs/All_States_historical_prices.xlsx
+++ b/outputs/All_States_historical_prices.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NSW" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QLD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIC" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="NSW" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="QLD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="VIC" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TAS" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6043,16 +6043,16 @@
         </is>
       </c>
       <c r="B274" s="3" t="n">
-        <v>71.2</v>
+        <v>70.36</v>
       </c>
       <c r="C274" s="3" t="n">
-        <v>74.36</v>
+        <v>71.44</v>
       </c>
       <c r="D274" s="3" t="n">
-        <v>71.2</v>
+        <v>70.36</v>
       </c>
       <c r="E274" s="3" t="n">
-        <v>74.36</v>
+        <v>71.44</v>
       </c>
       <c r="F274" s="4" t="inlineStr"/>
     </row>
@@ -11673,16 +11673,16 @@
         </is>
       </c>
       <c r="B274" s="3" t="n">
-        <v>65.23</v>
+        <v>62.64</v>
       </c>
       <c r="C274" s="3" t="n">
-        <v>65.02</v>
+        <v>61.19</v>
       </c>
       <c r="D274" s="3" t="n">
-        <v>65.23</v>
+        <v>62.64</v>
       </c>
       <c r="E274" s="3" t="n">
-        <v>65.02</v>
+        <v>61.19</v>
       </c>
       <c r="F274" s="4" t="inlineStr"/>
     </row>
@@ -17303,16 +17303,16 @@
         </is>
       </c>
       <c r="B274" s="3" t="n">
-        <v>41.17</v>
+        <v>44.74</v>
       </c>
       <c r="C274" s="3" t="n">
-        <v>44.39</v>
+        <v>44.69</v>
       </c>
       <c r="D274" s="3" t="n">
-        <v>41.17</v>
+        <v>44.74</v>
       </c>
       <c r="E274" s="3" t="n">
-        <v>44.39</v>
+        <v>44.69</v>
       </c>
       <c r="F274" s="4" t="inlineStr"/>
     </row>
@@ -22933,16 +22933,16 @@
         </is>
       </c>
       <c r="B274" s="3" t="n">
-        <v>43.95</v>
+        <v>52.8</v>
       </c>
       <c r="C274" s="3" t="n">
-        <v>35.84</v>
+        <v>40.82</v>
       </c>
       <c r="D274" s="3" t="n">
-        <v>43.95</v>
+        <v>52.8</v>
       </c>
       <c r="E274" s="3" t="n">
-        <v>35.84</v>
+        <v>40.82</v>
       </c>
       <c r="F274" s="4" t="inlineStr"/>
     </row>
@@ -28123,16 +28123,16 @@
         </is>
       </c>
       <c r="B252" s="3" t="n">
-        <v>88.23999999999999</v>
+        <v>91.04000000000001</v>
       </c>
       <c r="C252" s="3" t="n">
-        <v>88.52</v>
+        <v>90.94</v>
       </c>
       <c r="D252" s="3" t="n">
-        <v>88.23999999999999</v>
+        <v>91.04000000000001</v>
       </c>
       <c r="E252" s="3" t="n">
-        <v>88.52</v>
+        <v>90.94</v>
       </c>
       <c r="F252" s="4" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Update historical price analysis 2026-06
</commit_message>
<xml_diff>
--- a/outputs/All_States_historical_prices.xlsx
+++ b/outputs/All_States_historical_prices.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F275"/>
+  <dimension ref="A1:F276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6076,6 +6076,26 @@
       </c>
       <c r="F275" s="4" t="inlineStr"/>
     </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="n">
+        <v>82.01000000000001</v>
+      </c>
+      <c r="C276" s="3" t="n">
+        <v>87.43000000000001</v>
+      </c>
+      <c r="D276" s="3" t="n">
+        <v>82.01000000000001</v>
+      </c>
+      <c r="E276" s="3" t="n">
+        <v>87.43000000000001</v>
+      </c>
+      <c r="F276" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6087,7 +6107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F275"/>
+  <dimension ref="A1:F276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11706,6 +11726,26 @@
       </c>
       <c r="F275" s="4" t="inlineStr"/>
     </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="n">
+        <v>76.34</v>
+      </c>
+      <c r="C276" s="3" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="D276" s="3" t="n">
+        <v>76.34</v>
+      </c>
+      <c r="E276" s="3" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="F276" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11717,7 +11757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F275"/>
+  <dimension ref="A1:F276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17336,6 +17376,26 @@
       </c>
       <c r="F275" s="4" t="inlineStr"/>
     </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="n">
+        <v>64.77</v>
+      </c>
+      <c r="C276" s="3" t="n">
+        <v>73.73999999999999</v>
+      </c>
+      <c r="D276" s="3" t="n">
+        <v>64.77</v>
+      </c>
+      <c r="E276" s="3" t="n">
+        <v>73.73999999999999</v>
+      </c>
+      <c r="F276" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17347,7 +17407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F275"/>
+  <dimension ref="A1:F276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22966,6 +23026,26 @@
       </c>
       <c r="F275" s="4" t="inlineStr"/>
     </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="n">
+        <v>77.48999999999999</v>
+      </c>
+      <c r="C276" s="3" t="n">
+        <v>86.72</v>
+      </c>
+      <c r="D276" s="3" t="n">
+        <v>77.48999999999999</v>
+      </c>
+      <c r="E276" s="3" t="n">
+        <v>86.72</v>
+      </c>
+      <c r="F276" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22977,7 +23057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F253"/>
+  <dimension ref="A1:F254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28156,6 +28236,26 @@
       </c>
       <c r="F253" s="4" t="inlineStr"/>
     </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B254" s="3" t="n">
+        <v>96.14</v>
+      </c>
+      <c r="C254" s="3" t="n">
+        <v>100.08</v>
+      </c>
+      <c r="D254" s="3" t="n">
+        <v>96.14</v>
+      </c>
+      <c r="E254" s="3" t="n">
+        <v>100.08</v>
+      </c>
+      <c r="F254" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update historical price analysis 2026-07
</commit_message>
<xml_diff>
--- a/outputs/All_States_historical_prices.xlsx
+++ b/outputs/All_States_historical_prices.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F276"/>
+  <dimension ref="A1:F277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6096,6 +6096,26 @@
       </c>
       <c r="F276" s="4" t="inlineStr"/>
     </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="C277" s="3" t="n">
+        <v>86.92</v>
+      </c>
+      <c r="D277" s="3" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="E277" s="3" t="n">
+        <v>86.92</v>
+      </c>
+      <c r="F277" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6107,7 +6127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F276"/>
+  <dimension ref="A1:F277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11746,6 +11766,26 @@
       </c>
       <c r="F276" s="4" t="inlineStr"/>
     </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="C277" s="3" t="n">
+        <v>70.73</v>
+      </c>
+      <c r="D277" s="3" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="E277" s="3" t="n">
+        <v>70.73</v>
+      </c>
+      <c r="F277" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11757,7 +11797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F276"/>
+  <dimension ref="A1:F277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17396,6 +17436,26 @@
       </c>
       <c r="F276" s="4" t="inlineStr"/>
     </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="n">
+        <v>66.81</v>
+      </c>
+      <c r="C277" s="3" t="n">
+        <v>78.04000000000001</v>
+      </c>
+      <c r="D277" s="3" t="n">
+        <v>66.81</v>
+      </c>
+      <c r="E277" s="3" t="n">
+        <v>78.04000000000001</v>
+      </c>
+      <c r="F277" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17407,7 +17467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F276"/>
+  <dimension ref="A1:F277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23046,6 +23106,26 @@
       </c>
       <c r="F276" s="4" t="inlineStr"/>
     </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="n">
+        <v>125.73</v>
+      </c>
+      <c r="C277" s="3" t="n">
+        <v>152.96</v>
+      </c>
+      <c r="D277" s="3" t="n">
+        <v>125.73</v>
+      </c>
+      <c r="E277" s="3" t="n">
+        <v>152.96</v>
+      </c>
+      <c r="F277" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23057,7 +23137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F254"/>
+  <dimension ref="A1:F255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28256,6 +28336,26 @@
       </c>
       <c r="F254" s="4" t="inlineStr"/>
     </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B255" s="3" t="n">
+        <v>76.83</v>
+      </c>
+      <c r="C255" s="3" t="n">
+        <v>81.73</v>
+      </c>
+      <c r="D255" s="3" t="n">
+        <v>76.83</v>
+      </c>
+      <c r="E255" s="3" t="n">
+        <v>81.73</v>
+      </c>
+      <c r="F255" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>